<commit_message>
Tabla de cruce: las dudas, resueltas leyendo; quedan cuatro preguntas
Leidas las firmadas escaneadas donde habia versiones, parejas cruzadas o
dos hojas en un fichero. Lo resuelto va en resoluciones_tanda1.json y se
aplica al montar. La vigencia ya no se avisa.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/cruce_hojas_tanda1.xlsx
+++ b/docs/cruce_hojas_tanda1.xlsx
@@ -34,7 +34,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -63,7 +63,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00FFD966"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -79,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -97,6 +102,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1015,7 +1023,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>la firmada se llama "no vale/anulado"</t>
+          <t>RESUELTO LEYENDO: La firmada se llama 'no vale': hoja descartada por vosotros.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1232,14 +1240,14 @@
           <t>008</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>la misma enviada sirve a 2 firmadas; la lectura avisa de algo raro</t>
+          <t>RESUELTO LEYENDO: Cálculo estructural para FAIN. La otra firmada con la misma enviada (009) son instrucciones de facturación, no una hoja.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1317,14 +1325,14 @@
           <t>009</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>APARTAR</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>la misma enviada sirve a 2 firmadas; la lectura avisa de algo raro</t>
+          <t>RESUELTO LEYENDO: No es una hoja: 'INSTRUCCIONES FAIN FACTURAS'. Documento de facturación (como las órdenes de compra).</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1402,16 +1410,12 @@
           <t>010</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>más de 6 meses entre hoja y firma</t>
-        </is>
-      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="inlineStr">
         <is>
           <t>2025-01-13</t>
@@ -1574,14 +1578,14 @@
           <t>012</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>APARTAR</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>más de 6 meses entre hoja y firma; la misma enviada sirve a 2 firmadas; la lectura avisa de algo raro</t>
+          <t>RESUELTO LEYENDO: Copia en Google Docs de la firmada 013 (mismo nombre). Duplicado.</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1659,14 +1663,14 @@
           <t>013</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>más de 6 meses entre hoja y firma; la misma enviada sirve a 2 firmadas; la lectura avisa de algo raro</t>
+          <t>RESUELTO LEYENDO: La firmada de verdad (PDF); 012 era su copia en Google Docs.</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1913,14 +1917,14 @@
           <t>016</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>la lectura avisa de algo raro</t>
+          <t>RESUELTO LEYENDO: El texto cita la ordenanza de Madrid aunque es Fuenlabrada: es la plantilla. Importes correctos.</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -2002,14 +2006,14 @@
           <t>017</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>la lectura avisa de algo raro</t>
+          <t>RESUELTO LEYENDO: El fichero lleva pegada delante otra propuesta (Virgen del Camino 17, sin fecha ni firma). Solo cuenta la de AV MANCHA 15.</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -2095,14 +2099,14 @@
           <t>018</t>
         </is>
       </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>la lectura avisa de algo raro</t>
+          <t>RESUELTO LEYENDO: El texto cita subvenciones del Ayto. de Madrid aunque es Pozuelo: es la plantilla. Importes correctos.</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -2267,14 +2271,14 @@
           <t>020</t>
         </is>
       </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>la lectura avisa de algo raro</t>
+          <t>RESUELTO LEYENDO: El fichero tiene DOS hojas (proyecto y subvención), firmadas juntas: se vuelcan como dos hojas.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -2437,12 +2441,12 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>REVISAR</t>
+          <t>PREGUNTA</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>concepto sin casar con el catálogo</t>
+          <t>PARA TI: Rampa + remodelación de portal: el portal no tiene tipo en el catálogo.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -2602,12 +2606,12 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>REVISAR</t>
+          <t>PREGUNTA</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>la lectura avisa de algo raro</t>
+          <t>PARA TI: Firmada = enviada (16-10-2024). Dos precios ALTERNATIVOS: consulta previa 1.000 si no encargan el proyecto, o proyecto+licencia+DF+CFO 5.500 (y la consulta no se cobra).</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2683,14 +2687,14 @@
           <t>025</t>
         </is>
       </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>la hoja es POSTERIOR a la firmada; el documento se tocó DESPUÉS de llegar firmada; la misma enviada sirve a 2 firmadas</t>
+          <t>RESUELTO LEYENDO: Mal emparejada por el nombre. Su enviada no está en la carpeta, pero la firmada trae el texto: hoja a IBERLEAN (contrata), proyecto de ascensor + DR + DF, 5.000 + IVA, pago 1/3 firma, 1/3 proyecto, 1/3 CFO. Datos sacados de la firmada.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -2700,7 +2704,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2025-03-21</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -2710,7 +2714,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>comunidad</t>
+          <t>contrata: IBERLEAN ACCESIBILIDAD S.L.</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -2725,7 +2729,7 @@
         </is>
       </c>
       <c r="K27" s="2" t="n">
-        <v>850</v>
+        <v>5000</v>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
@@ -2853,14 +2857,14 @@
           <t>027</t>
         </is>
       </c>
-      <c r="B29" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>APARTAR</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>más de 6 meses entre hoja y firma</t>
+          <t>RESUELTO LEYENDO: No es una hoja: 'CODIGOS DE PEDIDO desglose'. Documento de facturación.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -3021,14 +3025,14 @@
           <t>029</t>
         </is>
       </c>
-      <c r="B31" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>la misma enviada sirve a 2 firmadas; la lectura avisa de algo raro</t>
+          <t>RESUELTO LEYENDO: La otra firmada con la misma enviada (030) es la orden de compra de Schindler.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -3109,14 +3113,14 @@
           <t>030</t>
         </is>
       </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>APARTAR</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>la misma enviada sirve a 2 firmadas; la lectura avisa de algo raro</t>
+          <t>RESUELTO LEYENDO: Orden de compra de Schindler: facturación, no hoja.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -3701,14 +3705,14 @@
           <t>037</t>
         </is>
       </c>
-      <c r="B39" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>concepto sin casar con el catálogo</t>
+          <t>RESUELTO LEYENDO: Descuento por cesión de CAES: se casa con el bloque de SATE + ASCENSOR CON CESION DE CAES.</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -4051,14 +4055,14 @@
           <t>041</t>
         </is>
       </c>
-      <c r="B43" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>la lectura avisa de algo raro</t>
+          <t>RESUELTO LEYENDO: El fichero tiene DOS hojas (proyecto y subvención), firmadas juntas: se vuelcan como dos hojas.</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -6262,14 +6266,14 @@
           <t>066</t>
         </is>
       </c>
-      <c r="B68" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>la misma enviada sirve a 2 firmadas</t>
+          <t>RESUELTO LEYENDO: Dos PDF firmados el mismo día de la misma hoja (con 067): se guardan los dos en la misma hoja.</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -6355,14 +6359,14 @@
           <t>067</t>
         </is>
       </c>
-      <c r="B69" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>la misma enviada sirve a 2 firmadas</t>
+          <t>RESUELTO LEYENDO: Dos PDF firmados el mismo día de la misma hoja (con 066): se guardan los dos en la misma hoja.</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -6534,14 +6538,14 @@
           <t>069</t>
         </is>
       </c>
-      <c r="B71" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>concepto sin casar con el catálogo</t>
+          <t>RESUELTO LEYENDO: Descuento por cesión de CAES (-8.600, total 10.200): bloque SATE CON CESION DE CAES.</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -6716,14 +6720,14 @@
           <t>071</t>
         </is>
       </c>
-      <c r="B73" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>más de 6 meses entre hoja y firma; la misma enviada sirve a 2 firmadas; la lectura avisa de algo raro</t>
+          <t>RESUELTO LEYENDO: El fichero tiene DOS hojas: esta firmada es la del PROYECTO (la de subvención es 072).</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -6801,14 +6805,14 @@
           <t>072</t>
         </is>
       </c>
-      <c r="B74" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>más de 6 meses entre hoja y firma; la misma enviada sirve a 2 firmadas; la lectura avisa de algo raro</t>
+          <t>RESUELTO LEYENDO: El fichero tiene DOS hojas: esta firmada es la de SUBVENCIÓN (la de proyecto es 071).</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -6886,14 +6890,14 @@
           <t>073</t>
         </is>
       </c>
-      <c r="B75" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>el documento se tocó DESPUÉS de llegar firmada</t>
+          <t>RESUELTO LEYENDO: Leída la firmada: 17/09/2025, ascensor 6.500 + envolvente con CAES 8.500 = 15.000. Es la misma versión aunque el documento se tocara después.</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -6988,12 +6992,12 @@
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>REVISAR</t>
+          <t>PREGUNTA</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>concepto sin casar con el catálogo</t>
+          <t>PARA TI: 'Proyecto para instalación de elevador' para IBERLEAN: ¿ascensor o plataforma?</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -7075,14 +7079,14 @@
           <t>075</t>
         </is>
       </c>
-      <c r="B77" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>más de 6 meses entre hoja y firma; la lectura avisa de algo raro</t>
+          <t>RESUELTO LEYENDO: El fichero tiene DOS hojas (proyecto y subvención), firmadas juntas: se vuelcan como dos hojas.</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -7161,16 +7165,12 @@
           <t>076</t>
         </is>
       </c>
-      <c r="B78" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
-        </is>
-      </c>
-      <c r="C78" s="2" t="inlineStr">
-        <is>
-          <t>más de 6 meses entre hoja y firma</t>
-        </is>
-      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr"/>
       <c r="D78" s="2" t="inlineStr">
         <is>
           <t>2025-11-05</t>
@@ -7621,14 +7621,14 @@
           <t>081</t>
         </is>
       </c>
-      <c r="B83" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>el documento se tocó DESPUÉS de llegar firmada; la misma enviada sirve a 2 firmadas; la lectura avisa de algo raro</t>
+          <t>RESUELTO LEYENDO: CSS de 08/01/2026. (La otra firmada que apuntaba aquí, 025, era otra hoja.)</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -8154,14 +8154,14 @@
           <t>087</t>
         </is>
       </c>
-      <c r="B89" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B89" s="7" t="inlineStr">
+        <is>
+          <t>ANULADA</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>la misma enviada sirve a 2 firmadas</t>
+          <t>RESUELTO LEYENDO: La firmada dice 'SIN EFECTO': la sustituyó la hoja de ascensor + SATE + subvención (122). Caso 4: se vuelca como anulada.</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
@@ -8523,14 +8523,14 @@
           <t>091</t>
         </is>
       </c>
-      <c r="B93" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>concepto sin casar con el catálogo</t>
+          <t>RESUELTO LEYENDO: 'Gestión de CAES' va dentro del precio del SATE: bloque SATE CON CESION DE CAES.</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
@@ -9146,14 +9146,14 @@
           <t>098</t>
         </is>
       </c>
-      <c r="B100" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>concepto sin casar con el catálogo</t>
+          <t>RESUELTO LEYENDO: Descuento por cesión de CAES (-17.570, total 8.500): bloque SATE CON CESION DE CAES.</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
@@ -9412,14 +9412,14 @@
           <t>101</t>
         </is>
       </c>
-      <c r="B103" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>la lectura avisa de algo raro</t>
+          <t>RESUELTO LEYENDO: La hoja dice 'UNANUME' (errata); la dirección buena es la de la opp.</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
@@ -9683,14 +9683,14 @@
           <t>104</t>
         </is>
       </c>
-      <c r="B106" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>hay otra versión en la carpeta</t>
+          <t>RESUELTO LEYENDO: Leída la firmada: 25/02/2026, 10.000 + 3,5%: es el documento original, no el 'Modificado'.</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -9785,14 +9785,14 @@
           <t>105</t>
         </is>
       </c>
-      <c r="B107" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>hay otra versión en la carpeta</t>
+          <t>RESUELTO LEYENDO: Leída la firmada: es del 11/03/2026, la versión 'Modificada' (v2). Mismo importe, 24.400 + 3,5%. Versiones: v1 25/02 enviada, v2 11/03 firmada.</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
@@ -9802,7 +9802,7 @@
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="F107" s="2" t="inlineStr">
@@ -10162,16 +10162,12 @@
           <t>109</t>
         </is>
       </c>
-      <c r="B111" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
-        </is>
-      </c>
-      <c r="C111" s="2" t="inlineStr">
-        <is>
-          <t>más de 6 meses entre hoja y firma</t>
-        </is>
-      </c>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr"/>
       <c r="D111" s="2" t="inlineStr">
         <is>
           <t>2026-04-08</t>
@@ -11257,14 +11253,14 @@
           <t>121</t>
         </is>
       </c>
-      <c r="B123" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B123" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>hay otra versión en la carpeta</t>
+          <t>RESUELTO LEYENDO: Leída la firmada: 25/02/2026, 10.000 + 3,5%, el original. Anotado a mano: aprobado en JG ordinaria 11-05-2026.</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
@@ -11359,14 +11355,14 @@
           <t>122</t>
         </is>
       </c>
-      <c r="B124" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B124" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>la misma enviada sirve a 2 firmadas</t>
+          <t>RESUELTO LEYENDO: Caso 4: hoja NUEVA que sustituye a la 087. Su enviada no está en la carpeta (salió de una adenda); datos leídos de la firmada: ascensor 6.940 + SATE 7.220 + subvención 1.980 fijo y 3,5% = 16.140. Trae lo ya abonado (5.450): eso es de facturación.</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
@@ -11409,7 +11405,7 @@
         </is>
       </c>
       <c r="K124" s="2" t="n">
-        <v>6940</v>
+        <v>16140</v>
       </c>
       <c r="L124" s="2" t="inlineStr">
         <is>
@@ -11456,14 +11452,14 @@
           <t>123</t>
         </is>
       </c>
-      <c r="B125" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B125" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>hay otra versión en la carpeta</t>
+          <t>RESUELTO LEYENDO: Leída la firmada: 28/05/2026, la versión 'modificado tras reunión' (v2). Mismos importes (proyecto 22.000; subvención 2.500 fijo + 3,5%); cambia el calendario de pagos. CIF con E (comunidad de bienes).</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
@@ -11473,7 +11469,7 @@
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="F125" s="2" t="inlineStr">
@@ -11921,14 +11917,14 @@
           <t>128</t>
         </is>
       </c>
-      <c r="B130" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>más de 6 meses entre hoja y firma</t>
+          <t>RESUELTO LEYENDO: Mal emparejada por el nombre. Su enviada es 'MODF ACEUCHAL 18 - 19/03/2026 - SUBV PRY PROP': subvención, tramo fijo 1.680 (1.980 tachado: descuento por IEE válida) + 3,5%.</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
@@ -11938,7 +11934,7 @@
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>2024-02-09</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="F130" s="2" t="inlineStr">
@@ -11967,7 +11963,7 @@
         </is>
       </c>
       <c r="K130" s="2" t="n">
-        <v>4000</v>
+        <v>1680</v>
       </c>
       <c r="L130" s="2" t="inlineStr">
         <is>
@@ -12362,14 +12358,14 @@
           <t>133</t>
         </is>
       </c>
-      <c r="B135" s="6" t="inlineStr">
-        <is>
-          <t>REVISAR</t>
+      <c r="B135" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>concepto sin casar con el catálogo</t>
+          <t>RESUELTO LEYENDO: El asesoramiento sobre ayudas va incluido en el precio del informe: no es línea aparte.</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
@@ -12543,12 +12539,12 @@
       </c>
       <c r="B137" s="6" t="inlineStr">
         <is>
-          <t>REVISAR</t>
+          <t>PREGUNTA</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>concepto sin casar con el catálogo</t>
+          <t>PARA TI: 'Mediciones y presupuesto ciego' (1.650): no hay bloque en el catálogo.</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Mediciones y ciego, Accesibilidad portal; tanda 1 de hojas cerrada
Bloque y tipo nuevos en el catalogo (aplicados en produccion). Sus
respuestas como reglas del cruce: elevador = plataforma, portal =
accesibilidad portal, precio alternativo = el proyecto.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/cruce_hojas_tanda1.xlsx
+++ b/docs/cruce_hojas_tanda1.xlsx
@@ -34,7 +34,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -63,11 +63,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFD966"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
@@ -84,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -102,9 +97,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2439,14 +2431,14 @@
           <t>022</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>PREGUNTA</t>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>PARA TI: Rampa + remodelación de portal: el portal no tiene tipo en el catálogo.</t>
+          <t>RESUELTO LEYENDO: Rampa + remodelación de portal: 'Accesibilidad portal' (Mónica: siempre hay rampa o escalón a salvar).</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -2471,14 +2463,10 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Rampa</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>remodelacion de portal</t>
-        </is>
-      </c>
+          <t>Rampa, Accesibilidad portal</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr">
         <is>
           <t>REDACCION PROYECTO: sin precio propio
@@ -2604,14 +2592,14 @@
           <t>024</t>
         </is>
       </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>PREGUNTA</t>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>PARA TI: Firmada = enviada (16-10-2024). Dos precios ALTERNATIVOS: consulta previa 1.000 si no encargan el proyecto, o proyecto+licencia+DF+CFO 5.500 (y la consulta no se cobra).</t>
+          <t>RESUELTO LEYENDO: Dos precios alternativos: se guarda el proyecto 5.500 como lo que se cobra; la consulta previa de 1.000 (solo si NO encargan el proyecto) queda como nota (Mónica).</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2649,7 +2637,9 @@
 CERTIFICADO FIN DE OBRA: sin precio propio</t>
         </is>
       </c>
-      <c r="K26" s="2" t="n"/>
+      <c r="K26" s="2" t="n">
+        <v>5500</v>
+      </c>
       <c r="L26" s="2" t="n"/>
       <c r="M26" s="2" t="inlineStr">
         <is>
@@ -6570,14 +6560,10 @@
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>SATE envolvente completa, Accesibilidad, Subvenciones, CAES</t>
-        </is>
-      </c>
-      <c r="I71" s="2" t="inlineStr">
-        <is>
-          <t>Rehabilitacion de Portal</t>
-        </is>
-      </c>
+          <t>SATE envolvente completa, Accesibilidad, Subvenciones, CAES, Accesibilidad portal</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr"/>
       <c r="J71" s="2" t="inlineStr">
         <is>
           <t>REDACCION PROYECTO: 14500 €
@@ -6990,14 +6976,14 @@
           <t>074</t>
         </is>
       </c>
-      <c r="B76" s="6" t="inlineStr">
-        <is>
-          <t>PREGUNTA</t>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>PARA TI: 'Proyecto para instalación de elevador' para IBERLEAN: ¿ascensor o plataforma?</t>
+          <t>RESUELTO LEYENDO: Elevador = plataforma elevadora = Plataforma (Mónica).</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -7020,12 +7006,12 @@
           <t>comunidad</t>
         </is>
       </c>
-      <c r="H76" s="2" t="inlineStr"/>
-      <c r="I76" s="2" t="inlineStr">
-        <is>
-          <t>Proyecto para instalación de elevador</t>
-        </is>
-      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr"/>
       <c r="J76" s="2" t="inlineStr">
         <is>
           <t>TOMA DE DATOS Y MODELADO 3D: sin precio propio
@@ -8154,7 +8140,7 @@
           <t>087</t>
         </is>
       </c>
-      <c r="B89" s="7" t="inlineStr">
+      <c r="B89" s="6" t="inlineStr">
         <is>
           <t>ANULADA</t>
         </is>
@@ -12537,14 +12523,14 @@
           <t>135</t>
         </is>
       </c>
-      <c r="B137" s="6" t="inlineStr">
-        <is>
-          <t>PREGUNTA</t>
+      <c r="B137" s="3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>PARA TI: 'Mediciones y presupuesto ciego' (1.650): no hay bloque en el catálogo.</t>
+          <t>RESUELTO LEYENDO: Bloque nuevo MEDICIONES Y CIEGO (Mónica, 6-oct).</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
@@ -12568,16 +12554,12 @@
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr"/>
-      <c r="I137" s="2" t="inlineStr">
-        <is>
-          <t>REDACCIÓN DE MEDICIONES Y PRESUPUESTO CIEGO</t>
-        </is>
-      </c>
+      <c r="I137" s="2" t="inlineStr"/>
       <c r="J137" s="2" t="inlineStr">
         <is>
           <t>TOMA DE DATOS Y MODELADO 3D: sin precio propio
 INFORME PERICIAL: sin precio propio
-SIN CASAR: sin precio propio</t>
+MEDICIONES Y CIEGO: sin precio propio</t>
         </is>
       </c>
       <c r="K137" s="2" t="n">
@@ -32715,7 +32697,7 @@
       </c>
       <c r="D733" s="2" t="inlineStr">
         <is>
-          <t>SIN CASAR</t>
+          <t>MEDICIONES Y CIEGO</t>
         </is>
       </c>
       <c r="E733" s="2" t="n"/>

</xml_diff>

<commit_message>
Tablas de cruce: quien genero la hoja segun el Excel de las automaticas, solo como cotejo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/cruce_hojas_tanda1.xlsx
+++ b/docs/cruce_hojas_tanda1.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conceptos" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cruce'!$A$1:$U$137</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cruce'!$A$1:$V$137</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Conceptos'!$A$1:$H$736</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U137"/>
+  <dimension ref="A1:V137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -485,9 +485,10 @@
     <col width="14" customWidth="1" min="16" max="16"/>
     <col width="35" customWidth="1" min="17" max="17"/>
     <col width="50" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="10" customWidth="1" min="20" max="20"/>
-    <col width="30" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="30" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -583,15 +584,20 @@
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
+          <t>Generada por (Excel, solo cotejo)</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
           <t>Código HE</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Opp</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>TU DECISIÓN</t>
         </is>
@@ -668,13 +674,14 @@
           <t>varios portales en una hoja (14 al 24); solo a éxito 2,5%</t>
         </is>
       </c>
-      <c r="S2" s="2" t="inlineStr">
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T2" s="2" t="inlineStr"/>
-      <c r="U2" s="4" t="inlineStr"/>
+      <c r="U2" s="2" t="inlineStr"/>
+      <c r="V2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -745,13 +752,14 @@
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr"/>
       <c r="R3" s="2" t="n"/>
-      <c r="S3" s="2" t="inlineStr">
+      <c r="S3" s="2" t="n"/>
+      <c r="T3" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T3" s="2" t="inlineStr"/>
-      <c r="U3" s="4" t="inlineStr"/>
+      <c r="U3" s="2" t="inlineStr"/>
+      <c r="V3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -823,13 +831,14 @@
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
       <c r="R4" s="2" t="n"/>
-      <c r="S4" s="2" t="inlineStr">
+      <c r="S4" s="2" t="n"/>
+      <c r="T4" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T4" s="2" t="inlineStr"/>
-      <c r="U4" s="4" t="inlineStr"/>
+      <c r="U4" s="2" t="inlineStr"/>
+      <c r="V4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -907,13 +916,14 @@
           <t>total = 1.500 fijo + 3% a éxito; la cabecera dice 'Proyecto para Rehabilitación de Envolvente Térmica' pero solo se cobra la tramitación de subvenciones; 'Otra Documentación Técnica' sin bloque</t>
         </is>
       </c>
-      <c r="S5" s="2" t="inlineStr">
+      <c r="S5" s="2" t="n"/>
+      <c r="T5" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T5" s="2" t="inlineStr"/>
-      <c r="U5" s="4" t="inlineStr"/>
+      <c r="U5" s="2" t="inlineStr"/>
+      <c r="V5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -994,13 +1004,14 @@
           <t>precio conjunto 5.900 sin desglose por concepto</t>
         </is>
       </c>
-      <c r="S6" s="2" t="inlineStr">
+      <c r="S6" s="2" t="n"/>
+      <c r="T6" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T6" s="2" t="inlineStr"/>
-      <c r="U6" s="4" t="inlineStr"/>
+      <c r="U6" s="2" t="inlineStr"/>
+      <c r="V6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1053,13 +1064,14 @@
           <t>sin texto</t>
         </is>
       </c>
-      <c r="S7" s="2" t="inlineStr">
+      <c r="S7" s="2" t="n"/>
+      <c r="T7" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T7" s="2" t="inlineStr"/>
-      <c r="U7" s="4" t="inlineStr"/>
+      <c r="U7" s="2" t="inlineStr"/>
+      <c r="V7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1136,13 +1148,14 @@
           <t>la línea de 3.760 agrupa toma de datos, modelado 3D, proyecto y dirección de obra; casada a REDACCION PROYECTO</t>
         </is>
       </c>
-      <c r="S8" s="2" t="inlineStr">
+      <c r="S8" s="2" t="n"/>
+      <c r="T8" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T8" s="2" t="inlineStr"/>
-      <c r="U8" s="4" t="inlineStr"/>
+      <c r="U8" s="2" t="inlineStr"/>
+      <c r="V8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1219,13 +1232,14 @@
           <t>solo a éxito 2,5%, sin importe fijo; incluye monetización por CAEs; 'Otra Documentación Técnica' sin bloque</t>
         </is>
       </c>
-      <c r="S9" s="2" t="inlineStr">
+      <c r="S9" s="2" t="n"/>
+      <c r="T9" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T9" s="2" t="inlineStr"/>
-      <c r="U9" s="4" t="inlineStr"/>
+      <c r="U9" s="2" t="inlineStr"/>
+      <c r="V9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1304,13 +1318,14 @@
           <t>texto idéntico a 009 (duplicado); pagador sin nombre, la casilla Nº pedido sugiere contrata</t>
         </is>
       </c>
-      <c r="S10" s="2" t="inlineStr">
+      <c r="S10" s="2" t="n"/>
+      <c r="T10" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T10" s="2" t="inlineStr"/>
-      <c r="U10" s="4" t="inlineStr"/>
+      <c r="U10" s="2" t="inlineStr"/>
+      <c r="V10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1389,13 +1404,14 @@
           <t>texto idéntico a 008 (duplicado); pagador sin nombre, la casilla Nº pedido sugiere contrata</t>
         </is>
       </c>
-      <c r="S11" s="2" t="inlineStr">
+      <c r="S11" s="2" t="n"/>
+      <c r="T11" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T11" s="2" t="inlineStr"/>
-      <c r="U11" s="4" t="inlineStr"/>
+      <c r="U11" s="2" t="inlineStr"/>
+      <c r="V11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1473,13 +1489,14 @@
           <t>proyecto + licencia + DF a precio conjunto de 2.500; accesibilidad en planta baja</t>
         </is>
       </c>
-      <c r="S12" s="2" t="inlineStr">
+      <c r="S12" s="2" t="n"/>
+      <c r="T12" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T12" s="2" t="inlineStr"/>
-      <c r="U12" s="4" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr"/>
+      <c r="V12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1557,13 +1574,14 @@
           <t>precio conjunto 1.980 para todo; subvenciones de accesibilidad y eficiencia juntas, casado al bloque genérico; sin cabecera de empresa</t>
         </is>
       </c>
-      <c r="S13" s="2" t="inlineStr">
+      <c r="S13" s="2" t="n"/>
+      <c r="T13" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T13" s="2" t="inlineStr"/>
-      <c r="U13" s="4" t="inlineStr"/>
+      <c r="U13" s="2" t="inlineStr"/>
+      <c r="V13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1642,13 +1660,14 @@
           <t>texto idéntico a 013 (duplicado); proyecto+licencia+DF+CFO a precio conjunto de 5.500; total 7.480 calculado (la hoja no da total)</t>
         </is>
       </c>
-      <c r="S14" s="2" t="inlineStr">
+      <c r="S14" s="2" t="n"/>
+      <c r="T14" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T14" s="2" t="inlineStr"/>
-      <c r="U14" s="4" t="inlineStr"/>
+      <c r="U14" s="2" t="inlineStr"/>
+      <c r="V14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1727,13 +1746,14 @@
           <t>texto idéntico a 012 (duplicado); proyecto+licencia+DF+CFO a precio conjunto de 5.500; total 7.480 calculado (la hoja no da total)</t>
         </is>
       </c>
-      <c r="S15" s="2" t="inlineStr">
+      <c r="S15" s="2" t="n"/>
+      <c r="T15" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T15" s="2" t="inlineStr"/>
-      <c r="U15" s="4" t="inlineStr"/>
+      <c r="U15" s="2" t="inlineStr"/>
+      <c r="V15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1811,13 +1831,14 @@
           <t>precio conjunto 2.500 sin desglose</t>
         </is>
       </c>
-      <c r="S16" s="2" t="inlineStr">
+      <c r="S16" s="2" t="n"/>
+      <c r="T16" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T16" s="2" t="inlineStr"/>
-      <c r="U16" s="4" t="inlineStr"/>
+      <c r="U16" s="2" t="inlineStr"/>
+      <c r="V16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1896,13 +1917,14 @@
           <t>dos precios conjuntos: 6.000 (proyecto+licencia+subvenciones) y 4.000 (DF+CSS); total 10.000 sumado</t>
         </is>
       </c>
-      <c r="S17" s="2" t="inlineStr">
+      <c r="S17" s="2" t="n"/>
+      <c r="T17" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T17" s="2" t="inlineStr"/>
-      <c r="U17" s="4" t="inlineStr"/>
+      <c r="U17" s="2" t="inlineStr"/>
+      <c r="V17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1985,13 +2007,14 @@
           <t>precio conjunto 3.100; el texto cita la Ordenanza y el Ayuntamiento de Madrid aunque el edificio está en Fuenlabrada (texto posiblemente copiado de otra hoja)</t>
         </is>
       </c>
-      <c r="S18" s="2" t="inlineStr">
+      <c r="S18" s="2" t="n"/>
+      <c r="T18" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T18" s="2" t="inlineStr"/>
-      <c r="U18" s="4" t="inlineStr"/>
+      <c r="U18" s="2" t="inlineStr"/>
+      <c r="V18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2079,13 +2102,14 @@
           <t>el fichero lleva antes otra propuesta sin fecha para C/ Virgen del Camino 17 Leganés (envolvente y cubierta, 9.763 € desglosados); solo la de AV MANCHA 15 tiene fecha y firma; resto de conceptos sin precio (11.000 conjunto); SATE fachada dudoso (dice envolvente)</t>
         </is>
       </c>
-      <c r="S19" s="2" t="inlineStr">
+      <c r="S19" s="2" t="n"/>
+      <c r="T19" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T19" s="2" t="inlineStr"/>
-      <c r="U19" s="4" t="inlineStr"/>
+      <c r="U19" s="2" t="inlineStr"/>
+      <c r="V19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2169,13 +2193,14 @@
           <t>precio conjunto 12.500; cita subvenciones del Ayuntamiento de Madrid aunque el edificio está en Pozuelo; pago ligado a consulta urbanística</t>
         </is>
       </c>
-      <c r="S20" s="2" t="inlineStr">
+      <c r="S20" s="2" t="n"/>
+      <c r="T20" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T20" s="2" t="inlineStr"/>
-      <c r="U20" s="4" t="inlineStr"/>
+      <c r="U20" s="2" t="inlineStr"/>
+      <c r="V20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2251,13 +2276,14 @@
           <t>solo DF y CSS de una obra de ascensor; el proyecto no está en esta hoja</t>
         </is>
       </c>
-      <c r="S21" s="2" t="inlineStr">
+      <c r="S21" s="2" t="n"/>
+      <c r="T21" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T21" s="2" t="inlineStr"/>
-      <c r="U21" s="4" t="inlineStr"/>
+      <c r="U21" s="2" t="inlineStr"/>
+      <c r="V21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2337,13 +2363,14 @@
           <t>dos hojas en un fichero (proyecto 5.650 y subvenciones 1.980); total 7.630 sumado; la línea de 3.910 agrupa toma de datos, proyecto, visado y dirección de obra</t>
         </is>
       </c>
-      <c r="S22" s="2" t="inlineStr">
+      <c r="S22" s="2" t="n"/>
+      <c r="T22" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T22" s="2" t="inlineStr"/>
-      <c r="U22" s="4" t="inlineStr"/>
+      <c r="U22" s="2" t="inlineStr"/>
+      <c r="V22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2419,13 +2446,14 @@
           <t>precio conjunto 2.400 DF+CSS; obra de ascensor con proyecto externo; en la casilla CIF pone la razón social</t>
         </is>
       </c>
-      <c r="S23" s="2" t="inlineStr">
+      <c r="S23" s="2" t="n"/>
+      <c r="T23" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T23" s="2" t="inlineStr"/>
-      <c r="U23" s="4" t="inlineStr"/>
+      <c r="U23" s="2" t="inlineStr"/>
+      <c r="V23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2507,13 +2535,14 @@
           <t>precio conjunto 2.500; incluye remodelación de portal</t>
         </is>
       </c>
-      <c r="S24" s="2" t="inlineStr">
+      <c r="S24" s="2" t="n"/>
+      <c r="T24" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T24" s="2" t="inlineStr"/>
-      <c r="U24" s="4" t="inlineStr"/>
+      <c r="U24" s="2" t="inlineStr"/>
+      <c r="V24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2580,13 +2609,14 @@
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr"/>
       <c r="R25" s="2" t="n"/>
-      <c r="S25" s="2" t="inlineStr">
+      <c r="S25" s="2" t="n"/>
+      <c r="T25" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T25" s="2" t="inlineStr"/>
-      <c r="U25" s="4" t="inlineStr"/>
+      <c r="U25" s="2" t="inlineStr"/>
+      <c r="V25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2665,13 +2695,14 @@
           <t>importes alternativos: consulta previa 1.000 (solo si no se encarga el proyecto) o proyecto+licencia+DF+CFO 5.500 conjunto (la consulta no se cobra); total null por ser alternativos</t>
         </is>
       </c>
-      <c r="S26" s="2" t="inlineStr">
+      <c r="S26" s="2" t="n"/>
+      <c r="T26" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T26" s="2" t="inlineStr"/>
-      <c r="U26" s="4" t="inlineStr"/>
+      <c r="U26" s="2" t="inlineStr"/>
+      <c r="V26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2752,11 +2783,16 @@
       <c r="R27" s="2" t="n"/>
       <c r="S27" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T27" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T27" s="2" t="inlineStr"/>
-      <c r="U27" s="4" t="inlineStr"/>
+      <c r="U27" s="2" t="inlineStr"/>
+      <c r="V27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2835,13 +2871,14 @@
           <t>precio conjunto 4.000; dirección con dos números (1-3)</t>
         </is>
       </c>
-      <c r="S28" s="2" t="inlineStr">
+      <c r="S28" s="2" t="n"/>
+      <c r="T28" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T28" s="2" t="inlineStr"/>
-      <c r="U28" s="4" t="inlineStr"/>
+      <c r="U28" s="2" t="inlineStr"/>
+      <c r="V28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2917,13 +2954,14 @@
       <c r="P29" s="2" t="inlineStr"/>
       <c r="Q29" s="2" t="inlineStr"/>
       <c r="R29" s="2" t="n"/>
-      <c r="S29" s="2" t="inlineStr">
+      <c r="S29" s="2" t="n"/>
+      <c r="T29" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T29" s="2" t="inlineStr"/>
-      <c r="U29" s="4" t="inlineStr"/>
+      <c r="U29" s="2" t="inlineStr"/>
+      <c r="V29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -3003,13 +3041,14 @@
           <t>PROYECTO Y DIRECCIÓN FACULTATIVA 3.753,40 conjunto (toma de datos, proyecto, licencia, DF y CFO)</t>
         </is>
       </c>
-      <c r="S30" s="2" t="inlineStr">
+      <c r="S30" s="2" t="n"/>
+      <c r="T30" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T30" s="2" t="inlineStr"/>
-      <c r="U30" s="4" t="inlineStr"/>
+      <c r="U30" s="2" t="inlineStr"/>
+      <c r="V30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -3091,13 +3130,14 @@
           <t>texto idéntico a 030 (duplicado); precio conjunto 3.600; 'cambio completo de dos ascensores' casado a Modificación asc. (dudoso)</t>
         </is>
       </c>
-      <c r="S31" s="2" t="inlineStr">
+      <c r="S31" s="2" t="n"/>
+      <c r="T31" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T31" s="2" t="inlineStr"/>
-      <c r="U31" s="4" t="inlineStr"/>
+      <c r="U31" s="2" t="inlineStr"/>
+      <c r="V31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -3179,13 +3219,14 @@
           <t>texto idéntico a 029 (duplicado); precio conjunto 3.600; 'cambio completo de dos ascensores' casado a Modificación asc. (dudoso)</t>
         </is>
       </c>
-      <c r="S32" s="2" t="inlineStr">
+      <c r="S32" s="2" t="n"/>
+      <c r="T32" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T32" s="2" t="inlineStr"/>
-      <c r="U32" s="4" t="inlineStr"/>
+      <c r="U32" s="2" t="inlineStr"/>
+      <c r="V32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -3260,13 +3301,14 @@
       </c>
       <c r="Q33" s="2" t="inlineStr"/>
       <c r="R33" s="2" t="n"/>
-      <c r="S33" s="2" t="inlineStr">
+      <c r="S33" s="2" t="n"/>
+      <c r="T33" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T33" s="2" t="inlineStr"/>
-      <c r="U33" s="4" t="inlineStr"/>
+      <c r="U33" s="2" t="inlineStr"/>
+      <c r="V33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3345,13 +3387,14 @@
           <t>proyecto+licencia+DF+CFO a precio conjunto de 3.500; en la casilla CIF pone la razón social</t>
         </is>
       </c>
-      <c r="S34" s="2" t="inlineStr">
+      <c r="S34" s="2" t="n"/>
+      <c r="T34" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T34" s="2" t="inlineStr"/>
-      <c r="U34" s="4" t="inlineStr"/>
+      <c r="U34" s="2" t="inlineStr"/>
+      <c r="V34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3430,13 +3473,14 @@
           <t>proyecto+licencia+DF+CFO a precio conjunto de 3.500; municipio mal escrito (MADIRD); en la casilla CIF pone la razón social</t>
         </is>
       </c>
-      <c r="S35" s="2" t="inlineStr">
+      <c r="S35" s="2" t="n"/>
+      <c r="T35" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T35" s="2" t="inlineStr"/>
-      <c r="U35" s="4" t="inlineStr"/>
+      <c r="U35" s="2" t="inlineStr"/>
+      <c r="V35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3511,13 +3555,14 @@
           <t>oferta especial de renovación consecutiva (no es primera presentación); sin cabecera de empresa</t>
         </is>
       </c>
-      <c r="S36" s="2" t="inlineStr">
+      <c r="S36" s="2" t="n"/>
+      <c r="T36" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T36" s="2" t="inlineStr"/>
-      <c r="U36" s="4" t="inlineStr"/>
+      <c r="U36" s="2" t="inlineStr"/>
+      <c r="V36" s="4" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3596,13 +3641,14 @@
           <t>Dirección sin municipio en la hoja (el título dice Madrid)</t>
         </is>
       </c>
-      <c r="S37" s="2" t="inlineStr">
+      <c r="S37" s="2" t="n"/>
+      <c r="T37" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T37" s="2" t="inlineStr"/>
-      <c r="U37" s="4" t="inlineStr"/>
+      <c r="U37" s="2" t="inlineStr"/>
+      <c r="V37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3683,13 +3729,14 @@
           <t>Precio conjunto: tramo fijo 2.225 para subvenciones + IEE + LEE, sin desglose</t>
         </is>
       </c>
-      <c r="S38" s="2" t="inlineStr">
+      <c r="S38" s="2" t="n"/>
+      <c r="T38" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T38" s="2" t="inlineStr"/>
-      <c r="U38" s="4" t="inlineStr"/>
+      <c r="U38" s="2" t="inlineStr"/>
+      <c r="V38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3776,13 +3823,14 @@
           <t>cabecera solo dice envolvente térmica pero el desglose cobra también proyecto de ascensor; honorarios rebajados a cambio de cesión de CAEs (descuento sin importe); subvenciones 'a éxito' pero con importe fijo 1.980</t>
         </is>
       </c>
-      <c r="S39" s="2" t="inlineStr">
+      <c r="S39" s="2" t="n"/>
+      <c r="T39" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T39" s="2" t="inlineStr"/>
-      <c r="U39" s="4" t="inlineStr"/>
+      <c r="U39" s="2" t="inlineStr"/>
+      <c r="V39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3855,13 +3903,14 @@
       </c>
       <c r="Q40" s="2" t="inlineStr"/>
       <c r="R40" s="2" t="n"/>
-      <c r="S40" s="2" t="inlineStr">
+      <c r="S40" s="2" t="n"/>
+      <c r="T40" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T40" s="2" t="inlineStr"/>
-      <c r="U40" s="4" t="inlineStr"/>
+      <c r="U40" s="2" t="inlineStr"/>
+      <c r="V40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3938,13 +3987,14 @@
           <t>Solo tramo variable 3,5%, sin tramo fijo; dirección sin municipio</t>
         </is>
       </c>
-      <c r="S41" s="2" t="inlineStr">
+      <c r="S41" s="2" t="n"/>
+      <c r="T41" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T41" s="2" t="inlineStr"/>
-      <c r="U41" s="4" t="inlineStr"/>
+      <c r="U41" s="2" t="inlineStr"/>
+      <c r="V41" s="4" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -4033,13 +4083,14 @@
           <t>Honorarios de proyecto 7.092 conjuntos sin desglose; IEE/LEE/CEE/consulta sin precio y no se sabe si van en proyecto o subvención; total_base = 7.092 + 1.980; título dice FAIN (posible ascensorista pagador)</t>
         </is>
       </c>
-      <c r="S42" s="2" t="inlineStr">
+      <c r="S42" s="2" t="n"/>
+      <c r="T42" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T42" s="2" t="inlineStr"/>
-      <c r="U42" s="4" t="inlineStr"/>
+      <c r="U42" s="2" t="inlineStr"/>
+      <c r="V42" s="4" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -4122,13 +4173,14 @@
           <t>dos hojas en un fichero (proyecto 5.900 a precio conjunto y subvenciones 1.980); total 7.880 sumado</t>
         </is>
       </c>
-      <c r="S43" s="2" t="inlineStr">
+      <c r="S43" s="2" t="n"/>
+      <c r="T43" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T43" s="2" t="inlineStr"/>
-      <c r="U43" s="4" t="inlineStr"/>
+      <c r="U43" s="2" t="inlineStr"/>
+      <c r="V43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -4207,13 +4259,14 @@
           <t>Es renovación de subvenciones (encargo previo)</t>
         </is>
       </c>
-      <c r="S44" s="2" t="inlineStr">
+      <c r="S44" s="2" t="n"/>
+      <c r="T44" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T44" s="2" t="inlineStr"/>
-      <c r="U44" s="4" t="inlineStr"/>
+      <c r="U44" s="2" t="inlineStr"/>
+      <c r="V44" s="4" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -4292,13 +4345,14 @@
           <t>La dirección no lleva municipio. El 3,5% variable solo aparece en la forma de pago, no en el total.</t>
         </is>
       </c>
-      <c r="S45" s="2" t="inlineStr">
+      <c r="S45" s="2" t="n"/>
+      <c r="T45" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T45" s="2" t="inlineStr"/>
-      <c r="U45" s="4" t="inlineStr"/>
+      <c r="U45" s="2" t="inlineStr"/>
+      <c r="V45" s="4" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -4377,13 +4431,14 @@
           <t>Dirección sin municipio en la hoja (el título dice Madrid)</t>
         </is>
       </c>
-      <c r="S46" s="2" t="inlineStr">
+      <c r="S46" s="2" t="n"/>
+      <c r="T46" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T46" s="2" t="inlineStr"/>
-      <c r="U46" s="4" t="inlineStr"/>
+      <c r="U46" s="2" t="inlineStr"/>
+      <c r="V46" s="4" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -4462,13 +4517,14 @@
           <t>Dirección sin municipio en la hoja (el título dice Madrid)</t>
         </is>
       </c>
-      <c r="S47" s="2" t="inlineStr">
+      <c r="S47" s="2" t="n"/>
+      <c r="T47" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T47" s="2" t="inlineStr"/>
-      <c r="U47" s="4" t="inlineStr"/>
+      <c r="U47" s="2" t="inlineStr"/>
+      <c r="V47" s="4" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -4551,13 +4607,14 @@
           <t>Proyecto 3.500 conjunto para redacción + licencia + fin de obra + DF, sin desglose; título menciona ROSERSESE</t>
         </is>
       </c>
-      <c r="S48" s="2" t="inlineStr">
+      <c r="S48" s="2" t="n"/>
+      <c r="T48" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T48" s="2" t="inlineStr"/>
-      <c r="U48" s="4" t="inlineStr"/>
+      <c r="U48" s="2" t="inlineStr"/>
+      <c r="V48" s="4" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -4637,13 +4694,14 @@
           <t>Precio conjunto 850 para IEE + CEE; no se reparte.</t>
         </is>
       </c>
-      <c r="S49" s="2" t="inlineStr">
+      <c r="S49" s="2" t="n"/>
+      <c r="T49" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T49" s="2" t="inlineStr"/>
-      <c r="U49" s="4" t="inlineStr"/>
+      <c r="U49" s="2" t="inlineStr"/>
+      <c r="V49" s="4" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -4722,13 +4780,14 @@
           <t>Dirección sin municipio en la hoja (el título dice Madrid)</t>
         </is>
       </c>
-      <c r="S50" s="2" t="inlineStr">
+      <c r="S50" s="2" t="n"/>
+      <c r="T50" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T50" s="2" t="inlineStr"/>
-      <c r="U50" s="4" t="inlineStr"/>
+      <c r="U50" s="2" t="inlineStr"/>
+      <c r="V50" s="4" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4804,13 +4863,14 @@
       </c>
       <c r="Q51" s="2" t="inlineStr"/>
       <c r="R51" s="2" t="n"/>
-      <c r="S51" s="2" t="inlineStr">
+      <c r="S51" s="2" t="n"/>
+      <c r="T51" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T51" s="2" t="inlineStr"/>
-      <c r="U51" s="4" t="inlineStr"/>
+      <c r="U51" s="2" t="inlineStr"/>
+      <c r="V51" s="4" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4889,13 +4949,14 @@
           <t>Dirección sin municipio en la hoja (el título dice Madrid)</t>
         </is>
       </c>
-      <c r="S52" s="2" t="inlineStr">
+      <c r="S52" s="2" t="n"/>
+      <c r="T52" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T52" s="2" t="inlineStr"/>
-      <c r="U52" s="4" t="inlineStr"/>
+      <c r="U52" s="2" t="inlineStr"/>
+      <c r="V52" s="4" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4975,13 +5036,14 @@
           <t>Precio conjunto 850 para IEE + CEE; no se reparte.</t>
         </is>
       </c>
-      <c r="S53" s="2" t="inlineStr">
+      <c r="S53" s="2" t="n"/>
+      <c r="T53" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T53" s="2" t="inlineStr"/>
-      <c r="U53" s="4" t="inlineStr"/>
+      <c r="U53" s="2" t="inlineStr"/>
+      <c r="V53" s="4" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -5069,13 +5131,14 @@
           <t>Honorarios de proyecto 5.900 conjuntos sin desglose; IEE/LEE/CEE sin precio, no se sabe si van en proyecto o subvención; subvención sin tramo variable; total_base = 5.900 + 1.980</t>
         </is>
       </c>
-      <c r="S54" s="2" t="inlineStr">
+      <c r="S54" s="2" t="n"/>
+      <c r="T54" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T54" s="2" t="inlineStr"/>
-      <c r="U54" s="4" t="inlineStr"/>
+      <c r="U54" s="2" t="inlineStr"/>
+      <c r="V54" s="4" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -5162,13 +5225,14 @@
           <t>Ascensor con derribo de escalera; proyecto 5.000 conjunto sin desglose; IEE/CEE sin precio, no se sabe si en proyecto o subvención; total_base = 5.000 + 1.980</t>
         </is>
       </c>
-      <c r="S55" s="2" t="inlineStr">
+      <c r="S55" s="2" t="n"/>
+      <c r="T55" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T55" s="2" t="inlineStr"/>
-      <c r="U55" s="4" t="inlineStr"/>
+      <c r="U55" s="2" t="inlineStr"/>
+      <c r="V55" s="4" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -5255,13 +5319,14 @@
           <t>Ascensor con derribo de escalera; proyecto 5.000 conjunto sin desglose; IEE/CEE sin precio, no se sabe si en proyecto o subvención; total_base = 5.000 + 1.980</t>
         </is>
       </c>
-      <c r="S56" s="2" t="inlineStr">
+      <c r="S56" s="2" t="n"/>
+      <c r="T56" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T56" s="2" t="inlineStr"/>
-      <c r="U56" s="4" t="inlineStr"/>
+      <c r="U56" s="2" t="inlineStr"/>
+      <c r="V56" s="4" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -5348,13 +5413,14 @@
           <t>Proyecto 5.000 es precio conjunto de toma de datos, proyecto, licencia, fin de obra, CSS y DF; IEE y CEE sin precio propio (no queda claro si van en proyecto o en subvención). Ascensor con derribo de escalera.</t>
         </is>
       </c>
-      <c r="S57" s="2" t="inlineStr">
+      <c r="S57" s="2" t="n"/>
+      <c r="T57" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T57" s="2" t="inlineStr"/>
-      <c r="U57" s="4" t="inlineStr"/>
+      <c r="U57" s="2" t="inlineStr"/>
+      <c r="V57" s="4" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -5433,13 +5499,14 @@
           <t>Dirección sin municipio en la hoja (el título dice Madrid)</t>
         </is>
       </c>
-      <c r="S58" s="2" t="inlineStr">
+      <c r="S58" s="2" t="n"/>
+      <c r="T58" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T58" s="2" t="inlineStr"/>
-      <c r="U58" s="4" t="inlineStr"/>
+      <c r="U58" s="2" t="inlineStr"/>
+      <c r="V58" s="4" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -5522,13 +5589,14 @@
           <t>Proyecto 3.500 conjunto para redacción + licencia + fin de obra + DF, sin desglose</t>
         </is>
       </c>
-      <c r="S59" s="2" t="inlineStr">
+      <c r="S59" s="2" t="n"/>
+      <c r="T59" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T59" s="2" t="inlineStr"/>
-      <c r="U59" s="4" t="inlineStr"/>
+      <c r="U59" s="2" t="inlineStr"/>
+      <c r="V59" s="4" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -5616,13 +5684,14 @@
           <t>La hoja dice 'ENVOLVENTE TÉRMICA' (título: SATE SIN CAES ROEN), casado como SATE envolvente completa; precio conjunto 8.360 incluida la subvención, sin tramo variable</t>
         </is>
       </c>
-      <c r="S60" s="2" t="inlineStr">
+      <c r="S60" s="2" t="n"/>
+      <c r="T60" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T60" s="2" t="inlineStr"/>
-      <c r="U60" s="4" t="inlineStr"/>
+      <c r="U60" s="2" t="inlineStr"/>
+      <c r="V60" s="4" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -5712,13 +5781,14 @@
           <t>Precio conjunto 10.000 para todo; no se reparte. 'Envolvente térmica' casado como SATE envolvente completa (la hoja no dice SATE, solo el título).</t>
         </is>
       </c>
-      <c r="S61" s="2" t="inlineStr">
+      <c r="S61" s="2" t="n"/>
+      <c r="T61" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T61" s="2" t="inlineStr"/>
-      <c r="U61" s="4" t="inlineStr"/>
+      <c r="U61" s="2" t="inlineStr"/>
+      <c r="V61" s="4" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -5801,13 +5871,14 @@
           <t>Proyecto 3.500 conjunto para redacción + licencia + fin de obra + DF, sin desglose</t>
         </is>
       </c>
-      <c r="S62" s="2" t="inlineStr">
+      <c r="S62" s="2" t="n"/>
+      <c r="T62" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T62" s="2" t="inlineStr"/>
-      <c r="U62" s="4" t="inlineStr"/>
+      <c r="U62" s="2" t="inlineStr"/>
+      <c r="V62" s="4" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -5883,13 +5954,14 @@
       </c>
       <c r="Q63" s="2" t="inlineStr"/>
       <c r="R63" s="2" t="n"/>
-      <c r="S63" s="2" t="inlineStr">
+      <c r="S63" s="2" t="n"/>
+      <c r="T63" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T63" s="2" t="inlineStr"/>
-      <c r="U63" s="4" t="inlineStr"/>
+      <c r="U63" s="2" t="inlineStr"/>
+      <c r="V63" s="4" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -5973,13 +6045,14 @@
           <t>La hoja dice 'SALVAESCALERAS', casado como Plataforma; arquitectura 2.500 conjunta sin desglose; CSS sin forma de pago propia</t>
         </is>
       </c>
-      <c r="S64" s="2" t="inlineStr">
+      <c r="S64" s="2" t="n"/>
+      <c r="T64" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T64" s="2" t="inlineStr"/>
-      <c r="U64" s="4" t="inlineStr"/>
+      <c r="U64" s="2" t="inlineStr"/>
+      <c r="V64" s="4" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -6062,13 +6135,14 @@
           <t>Sustitución de 7 ascensores casado como Modificación asc. Precio conjunto 14.000; no se reparte.</t>
         </is>
       </c>
-      <c r="S65" s="2" t="inlineStr">
+      <c r="S65" s="2" t="n"/>
+      <c r="T65" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T65" s="2" t="inlineStr"/>
-      <c r="U65" s="4" t="inlineStr"/>
+      <c r="U65" s="2" t="inlineStr"/>
+      <c r="V65" s="4" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -6155,13 +6229,14 @@
           <t>Precio conjunto 4.500 incluida la subvención (que tiene forma de pago propia pero sin importe propio)</t>
         </is>
       </c>
-      <c r="S66" s="2" t="inlineStr">
+      <c r="S66" s="2" t="n"/>
+      <c r="T66" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T66" s="2" t="inlineStr"/>
-      <c r="U66" s="4" t="inlineStr"/>
+      <c r="U66" s="2" t="inlineStr"/>
+      <c r="V66" s="4" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -6244,13 +6319,14 @@
           <t>Sustitución de 7 ascensores, casado como Modificación asc.; precio conjunto 7.000</t>
         </is>
       </c>
-      <c r="S67" s="2" t="inlineStr">
+      <c r="S67" s="2" t="n"/>
+      <c r="T67" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T67" s="2" t="inlineStr"/>
-      <c r="U67" s="4" t="inlineStr"/>
+      <c r="U67" s="2" t="inlineStr"/>
+      <c r="V67" s="4" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -6337,13 +6413,14 @@
           <t>Proyecto 3.500 conjunto para redacción + licencia + fin de obra + DF, sin desglose</t>
         </is>
       </c>
-      <c r="S68" s="2" t="inlineStr">
+      <c r="S68" s="2" t="n"/>
+      <c r="T68" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T68" s="2" t="inlineStr"/>
-      <c r="U68" s="4" t="inlineStr"/>
+      <c r="U68" s="2" t="inlineStr"/>
+      <c r="V68" s="4" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -6430,13 +6507,14 @@
           <t>Proyecto 3.500 es precio conjunto de proyecto, licencia, fin de obra y DF; no se reparte.</t>
         </is>
       </c>
-      <c r="S69" s="2" t="inlineStr">
+      <c r="S69" s="2" t="n"/>
+      <c r="T69" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T69" s="2" t="inlineStr"/>
-      <c r="U69" s="4" t="inlineStr"/>
+      <c r="U69" s="2" t="inlineStr"/>
+      <c r="V69" s="4" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -6516,13 +6594,14 @@
           <t>Precio conjunto 2.225 para subvención + IEE, sin desglose</t>
         </is>
       </c>
-      <c r="S70" s="2" t="inlineStr">
+      <c r="S70" s="2" t="n"/>
+      <c r="T70" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T70" s="2" t="inlineStr"/>
-      <c r="U70" s="4" t="inlineStr"/>
+      <c r="U70" s="2" t="inlineStr"/>
+      <c r="V70" s="4" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -6609,13 +6688,14 @@
           <t>los conceptos suman 18.880 pero la hoja dice 18.800 sin descuento; descuento de 8.600 por cesión de CAES (total con descuento 10.200, condicionado a firmar la cesión); además 3,5% a éxito en subvenciones; licencia, CEE y DF descritos sin precio propio</t>
         </is>
       </c>
-      <c r="S71" s="2" t="inlineStr">
+      <c r="S71" s="2" t="n"/>
+      <c r="T71" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T71" s="2" t="inlineStr"/>
-      <c r="U71" s="4" t="inlineStr"/>
+      <c r="U71" s="2" t="inlineStr"/>
+      <c r="V71" s="4" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -6694,13 +6774,14 @@
           <t>Estudio técnico de sustitución de viga estructural: se describe como memoria técnica + planos para DR, dudoso entre MEMORIA TECNICA e INFORME PERICIAL; título dice FAIN (posible ascensorista pagador)</t>
         </is>
       </c>
-      <c r="S72" s="2" t="inlineStr">
+      <c r="S72" s="2" t="n"/>
+      <c r="T72" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T72" s="2" t="inlineStr"/>
-      <c r="U72" s="4" t="inlineStr"/>
+      <c r="U72" s="2" t="inlineStr"/>
+      <c r="V72" s="4" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -6779,13 +6860,14 @@
           <t>texto idéntico a 072 (duplicado); dos hojas en un fichero (proyecto 6.000 y subvenciones 1.980); total 7.980 sumado; la línea de 4.260 agrupa toma de datos, proyecto, visado y dirección de obra</t>
         </is>
       </c>
-      <c r="S73" s="2" t="inlineStr">
+      <c r="S73" s="2" t="n"/>
+      <c r="T73" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T73" s="2" t="inlineStr"/>
-      <c r="U73" s="4" t="inlineStr"/>
+      <c r="U73" s="2" t="inlineStr"/>
+      <c r="V73" s="4" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -6864,13 +6946,14 @@
           <t>texto idéntico a 071 (duplicado); dos hojas en un fichero (proyecto 6.000 y subvenciones 1.980); total 7.980 sumado; la línea de 4.260 agrupa toma de datos, proyecto, visado y dirección de obra</t>
         </is>
       </c>
-      <c r="S74" s="2" t="inlineStr">
+      <c r="S74" s="2" t="n"/>
+      <c r="T74" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T74" s="2" t="inlineStr"/>
-      <c r="U74" s="4" t="inlineStr"/>
+      <c r="U74" s="2" t="inlineStr"/>
+      <c r="V74" s="4" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -6965,13 +7048,14 @@
           <t>Envolvente térmica casada como SATE; SATE 8.500 tras descuento por CAES de 6.430 sobre 14.930 (proyecto 11.000 + LE 1.300 + IEE 650 + subvención 1.980); la línea de 8.500 pone 'iva' sin '+'; ascensor 6.500 aparte; dudoso si el bloque es SATE + ASCENSOR CON CESION DE CAES</t>
         </is>
       </c>
-      <c r="S75" s="2" t="inlineStr">
+      <c r="S75" s="2" t="n"/>
+      <c r="T75" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T75" s="2" t="inlineStr"/>
-      <c r="U75" s="4" t="inlineStr"/>
+      <c r="U75" s="2" t="inlineStr"/>
+      <c r="V75" s="4" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -7054,13 +7138,14 @@
           <t>precio conjunto 3.736; 'elevador' sin casar (ascensor o plataforma); el conforme dice 'cliente', no consta que sea la comunidad</t>
         </is>
       </c>
-      <c r="S76" s="2" t="inlineStr">
+      <c r="S76" s="2" t="n"/>
+      <c r="T76" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T76" s="2" t="inlineStr"/>
-      <c r="U76" s="4" t="inlineStr"/>
+      <c r="U76" s="2" t="inlineStr"/>
+      <c r="V76" s="4" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -7140,13 +7225,14 @@
           <t>dos hojas en un fichero (proyecto 6.000 y subvenciones 1.980); total 7.980 sumado; la línea de 4.260 agrupa toma de datos, proyecto, visado y dirección de obra</t>
         </is>
       </c>
-      <c r="S77" s="2" t="inlineStr">
+      <c r="S77" s="2" t="n"/>
+      <c r="T77" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T77" s="2" t="inlineStr"/>
-      <c r="U77" s="4" t="inlineStr"/>
+      <c r="U77" s="2" t="inlineStr"/>
+      <c r="V77" s="4" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -7218,13 +7304,14 @@
       <c r="P78" s="2" t="inlineStr"/>
       <c r="Q78" s="2" t="inlineStr"/>
       <c r="R78" s="2" t="n"/>
-      <c r="S78" s="2" t="inlineStr">
+      <c r="S78" s="2" t="n"/>
+      <c r="T78" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T78" s="2" t="inlineStr"/>
-      <c r="U78" s="4" t="inlineStr"/>
+      <c r="U78" s="2" t="inlineStr"/>
+      <c r="V78" s="4" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -7313,13 +7400,14 @@
           <t>Importes por concepto son SIN descuento (suman 32.910); descuento por cesión de CAES -15.910 deja total 17.000. Encaja con bloque SATE CON CESION DE CAES. LEE con precio pero no está en el desglose; CEE en desglose sin precio. 'Envolvente térmica' casado como SATE envolvente completa.</t>
         </is>
       </c>
-      <c r="S79" s="2" t="inlineStr">
+      <c r="S79" s="2" t="n"/>
+      <c r="T79" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T79" s="2" t="inlineStr"/>
-      <c r="U79" s="4" t="inlineStr"/>
+      <c r="U79" s="2" t="inlineStr"/>
+      <c r="V79" s="4" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -7408,11 +7496,16 @@
       </c>
       <c r="S80" s="2" t="inlineStr">
         <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="T80" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T80" s="2" t="inlineStr"/>
-      <c r="U80" s="4" t="inlineStr"/>
+      <c r="U80" s="2" t="inlineStr"/>
+      <c r="V80" s="4" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -7501,13 +7594,14 @@
           <t>La hoja dice 'ENVOLVENTE TÉRMICA' (título: PRY SATE), casado como SATE envolvente completa; proyecto 9.800 conjunto; IEE/LEE/CEE sin precio; total_base = 9.800 + 1.980</t>
         </is>
       </c>
-      <c r="S81" s="2" t="inlineStr">
+      <c r="S81" s="2" t="n"/>
+      <c r="T81" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T81" s="2" t="inlineStr"/>
-      <c r="U81" s="4" t="inlineStr"/>
+      <c r="U81" s="2" t="inlineStr"/>
+      <c r="V81" s="4" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -7598,11 +7692,16 @@
       </c>
       <c r="S82" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T82" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T82" s="2" t="inlineStr"/>
-      <c r="U82" s="4" t="inlineStr"/>
+      <c r="U82" s="2" t="inlineStr"/>
+      <c r="V82" s="4" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -7687,11 +7786,16 @@
       </c>
       <c r="S83" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T83" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T83" s="2" t="inlineStr"/>
-      <c r="U83" s="4" t="inlineStr"/>
+      <c r="U83" s="2" t="inlineStr"/>
+      <c r="V83" s="4" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -7781,11 +7885,16 @@
       </c>
       <c r="S84" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T84" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T84" s="2" t="inlineStr"/>
-      <c r="U84" s="4" t="inlineStr"/>
+      <c r="U84" s="2" t="inlineStr"/>
+      <c r="V84" s="4" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -7862,11 +7971,16 @@
       <c r="R85" s="2" t="n"/>
       <c r="S85" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T85" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T85" s="2" t="inlineStr"/>
-      <c r="U85" s="4" t="inlineStr"/>
+      <c r="U85" s="2" t="inlineStr"/>
+      <c r="V85" s="4" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -7951,11 +8065,16 @@
       </c>
       <c r="S86" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T86" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T86" s="2" t="inlineStr"/>
-      <c r="U86" s="4" t="inlineStr"/>
+      <c r="U86" s="2" t="inlineStr"/>
+      <c r="V86" s="4" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -8036,11 +8155,16 @@
       </c>
       <c r="S87" s="2" t="inlineStr">
         <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="T87" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T87" s="2" t="inlineStr"/>
-      <c r="U87" s="4" t="inlineStr"/>
+      <c r="U87" s="2" t="inlineStr"/>
+      <c r="V87" s="4" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -8131,11 +8255,16 @@
       </c>
       <c r="S88" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T88" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T88" s="2" t="inlineStr"/>
-      <c r="U88" s="4" t="inlineStr"/>
+      <c r="U88" s="2" t="inlineStr"/>
+      <c r="V88" s="4" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -8228,11 +8357,16 @@
       </c>
       <c r="S89" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T89" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T89" s="2" t="inlineStr"/>
-      <c r="U89" s="4" t="inlineStr"/>
+      <c r="U89" s="2" t="inlineStr"/>
+      <c r="V89" s="4" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -8321,11 +8455,16 @@
       </c>
       <c r="S90" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T90" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T90" s="2" t="inlineStr"/>
-      <c r="U90" s="4" t="inlineStr"/>
+      <c r="U90" s="2" t="inlineStr"/>
+      <c r="V90" s="4" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -8415,11 +8554,16 @@
       </c>
       <c r="S91" s="2" t="inlineStr">
         <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="T91" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T91" s="2" t="inlineStr"/>
-      <c r="U91" s="4" t="inlineStr"/>
+      <c r="U91" s="2" t="inlineStr"/>
+      <c r="V91" s="4" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -8500,11 +8644,16 @@
       </c>
       <c r="S92" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T92" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T92" s="2" t="inlineStr"/>
-      <c r="U92" s="4" t="inlineStr"/>
+      <c r="U92" s="2" t="inlineStr"/>
+      <c r="V92" s="4" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -8599,11 +8748,16 @@
       </c>
       <c r="S93" s="2" t="inlineStr">
         <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="T93" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T93" s="2" t="inlineStr"/>
-      <c r="U93" s="4" t="inlineStr"/>
+      <c r="U93" s="2" t="inlineStr"/>
+      <c r="V93" s="4" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -8685,11 +8839,16 @@
       <c r="R94" s="2" t="n"/>
       <c r="S94" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T94" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T94" s="2" t="inlineStr"/>
-      <c r="U94" s="4" t="inlineStr"/>
+      <c r="U94" s="2" t="inlineStr"/>
+      <c r="V94" s="4" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -8775,11 +8934,16 @@
       </c>
       <c r="S95" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T95" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T95" s="2" t="inlineStr"/>
-      <c r="U95" s="4" t="inlineStr"/>
+      <c r="U95" s="2" t="inlineStr"/>
+      <c r="V95" s="4" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -8861,11 +9025,16 @@
       <c r="R96" s="2" t="n"/>
       <c r="S96" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T96" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T96" s="2" t="inlineStr"/>
-      <c r="U96" s="4" t="inlineStr"/>
+      <c r="U96" s="2" t="inlineStr"/>
+      <c r="V96" s="4" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -8947,11 +9116,16 @@
       <c r="R97" s="2" t="n"/>
       <c r="S97" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T97" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T97" s="2" t="inlineStr"/>
-      <c r="U97" s="4" t="inlineStr"/>
+      <c r="U97" s="2" t="inlineStr"/>
+      <c r="V97" s="4" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -9033,11 +9207,16 @@
       <c r="R98" s="2" t="n"/>
       <c r="S98" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T98" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T98" s="2" t="inlineStr"/>
-      <c r="U98" s="4" t="inlineStr"/>
+      <c r="U98" s="2" t="inlineStr"/>
+      <c r="V98" s="4" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -9123,11 +9302,16 @@
       </c>
       <c r="S99" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T99" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T99" s="2" t="inlineStr"/>
-      <c r="U99" s="4" t="inlineStr"/>
+      <c r="U99" s="2" t="inlineStr"/>
+      <c r="V99" s="4" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -9221,13 +9405,14 @@
           <t>Total sin descuento 26.070 (cuadra); descuento por cesión de CAES -17.570 deja 8.500 (posible bloque SATE CON CESION DE CAES); 'envolvente térmica' asimilada a SATE envolvente completa; CEE listado sin precio</t>
         </is>
       </c>
-      <c r="S100" s="2" t="inlineStr">
+      <c r="S100" s="2" t="n"/>
+      <c r="T100" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T100" s="2" t="inlineStr"/>
-      <c r="U100" s="4" t="inlineStr"/>
+      <c r="U100" s="2" t="inlineStr"/>
+      <c r="V100" s="4" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -9308,11 +9493,16 @@
       <c r="R101" s="2" t="n"/>
       <c r="S101" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T101" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T101" s="2" t="inlineStr"/>
-      <c r="U101" s="4" t="inlineStr"/>
+      <c r="U101" s="2" t="inlineStr"/>
+      <c r="V101" s="4" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -9389,11 +9579,16 @@
       <c r="R102" s="2" t="n"/>
       <c r="S102" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T102" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T102" s="2" t="inlineStr"/>
-      <c r="U102" s="4" t="inlineStr"/>
+      <c r="U102" s="2" t="inlineStr"/>
+      <c r="V102" s="4" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -9478,11 +9673,16 @@
       </c>
       <c r="S103" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T103" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T103" s="2" t="inlineStr"/>
-      <c r="U103" s="4" t="inlineStr"/>
+      <c r="U103" s="2" t="inlineStr"/>
+      <c r="V103" s="4" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -9573,11 +9773,16 @@
       </c>
       <c r="S104" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T104" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T104" s="2" t="inlineStr"/>
-      <c r="U104" s="4" t="inlineStr"/>
+      <c r="U104" s="2" t="inlineStr"/>
+      <c r="V104" s="4" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -9660,11 +9865,16 @@
       </c>
       <c r="S105" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T105" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T105" s="2" t="inlineStr"/>
-      <c r="U105" s="4" t="inlineStr"/>
+      <c r="U105" s="2" t="inlineStr"/>
+      <c r="V105" s="4" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -9762,11 +9972,16 @@
       </c>
       <c r="S106" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T106" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T106" s="2" t="inlineStr"/>
-      <c r="U106" s="4" t="inlineStr"/>
+      <c r="U106" s="2" t="inlineStr"/>
+      <c r="V106" s="4" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -9864,11 +10079,16 @@
       </c>
       <c r="S107" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T107" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T107" s="2" t="inlineStr"/>
-      <c r="U107" s="4" t="inlineStr"/>
+      <c r="U107" s="2" t="inlineStr"/>
+      <c r="V107" s="4" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -9957,11 +10177,16 @@
       </c>
       <c r="S108" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T108" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T108" s="2" t="inlineStr"/>
-      <c r="U108" s="4" t="inlineStr"/>
+      <c r="U108" s="2" t="inlineStr"/>
+      <c r="V108" s="4" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -10049,11 +10274,16 @@
       </c>
       <c r="S109" s="2" t="inlineStr">
         <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="T109" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T109" s="2" t="inlineStr"/>
-      <c r="U109" s="4" t="inlineStr"/>
+      <c r="U109" s="2" t="inlineStr"/>
+      <c r="V109" s="4" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -10139,11 +10369,16 @@
       </c>
       <c r="S110" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T110" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T110" s="2" t="inlineStr"/>
-      <c r="U110" s="4" t="inlineStr"/>
+      <c r="U110" s="2" t="inlineStr"/>
+      <c r="V110" s="4" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -10230,13 +10465,14 @@
           <t>Proyecto 6.500 precio conjunto (pago 4.900 + 1.600 DF); IEE y CEE sin precio propio. Subvención limitada a una presentación por entidad (CAM y Ayto).</t>
         </is>
       </c>
-      <c r="S111" s="2" t="inlineStr">
+      <c r="S111" s="2" t="n"/>
+      <c r="T111" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T111" s="2" t="inlineStr"/>
-      <c r="U111" s="4" t="inlineStr"/>
+      <c r="U111" s="2" t="inlineStr"/>
+      <c r="V111" s="4" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -10318,11 +10554,16 @@
       <c r="R112" s="2" t="n"/>
       <c r="S112" s="2" t="inlineStr">
         <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="T112" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T112" s="2" t="inlineStr"/>
-      <c r="U112" s="4" t="inlineStr"/>
+      <c r="U112" s="2" t="inlineStr"/>
+      <c r="V112" s="4" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -10408,11 +10649,16 @@
       </c>
       <c r="S113" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T113" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T113" s="2" t="inlineStr"/>
-      <c r="U113" s="4" t="inlineStr"/>
+      <c r="U113" s="2" t="inlineStr"/>
+      <c r="V113" s="4" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -10494,11 +10740,16 @@
       <c r="R114" s="2" t="n"/>
       <c r="S114" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T114" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T114" s="2" t="inlineStr"/>
-      <c r="U114" s="4" t="inlineStr"/>
+      <c r="U114" s="2" t="inlineStr"/>
+      <c r="V114" s="4" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -10584,11 +10835,16 @@
       </c>
       <c r="S115" s="2" t="inlineStr">
         <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="T115" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T115" s="2" t="inlineStr"/>
-      <c r="U115" s="4" t="inlineStr"/>
+      <c r="U115" s="2" t="inlineStr"/>
+      <c r="V115" s="4" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -10674,11 +10930,16 @@
       </c>
       <c r="S116" s="2" t="inlineStr">
         <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="T116" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T116" s="2" t="inlineStr"/>
-      <c r="U116" s="4" t="inlineStr"/>
+      <c r="U116" s="2" t="inlineStr"/>
+      <c r="V116" s="4" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -10755,11 +11016,16 @@
       <c r="R117" s="2" t="n"/>
       <c r="S117" s="2" t="inlineStr">
         <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="T117" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T117" s="2" t="inlineStr"/>
-      <c r="U117" s="4" t="inlineStr"/>
+      <c r="U117" s="2" t="inlineStr"/>
+      <c r="V117" s="4" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -10850,11 +11116,16 @@
       </c>
       <c r="S118" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T118" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T118" s="2" t="inlineStr"/>
-      <c r="U118" s="4" t="inlineStr"/>
+      <c r="U118" s="2" t="inlineStr"/>
+      <c r="V118" s="4" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -10945,11 +11216,16 @@
       </c>
       <c r="S119" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T119" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T119" s="2" t="inlineStr"/>
-      <c r="U119" s="4" t="inlineStr"/>
+      <c r="U119" s="2" t="inlineStr"/>
+      <c r="V119" s="4" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -11040,11 +11316,16 @@
       </c>
       <c r="S120" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T120" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T120" s="2" t="inlineStr"/>
-      <c r="U120" s="4" t="inlineStr"/>
+      <c r="U120" s="2" t="inlineStr"/>
+      <c r="V120" s="4" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -11135,11 +11416,16 @@
       </c>
       <c r="S121" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T121" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T121" s="2" t="inlineStr"/>
-      <c r="U121" s="4" t="inlineStr"/>
+      <c r="U121" s="2" t="inlineStr"/>
+      <c r="V121" s="4" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -11230,11 +11516,16 @@
       </c>
       <c r="S122" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T122" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T122" s="2" t="inlineStr"/>
-      <c r="U122" s="4" t="inlineStr"/>
+      <c r="U122" s="2" t="inlineStr"/>
+      <c r="V122" s="4" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -11332,11 +11623,16 @@
       </c>
       <c r="S123" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T123" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T123" s="2" t="inlineStr"/>
-      <c r="U123" s="4" t="inlineStr"/>
+      <c r="U123" s="2" t="inlineStr"/>
+      <c r="V123" s="4" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -11429,11 +11725,16 @@
       </c>
       <c r="S124" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T124" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T124" s="2" t="inlineStr"/>
-      <c r="U124" s="4" t="inlineStr"/>
+      <c r="U124" s="2" t="inlineStr"/>
+      <c r="V124" s="4" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -11530,11 +11831,16 @@
       </c>
       <c r="S125" s="2" t="inlineStr">
         <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="T125" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T125" s="2" t="inlineStr"/>
-      <c r="U125" s="4" t="inlineStr"/>
+      <c r="U125" s="2" t="inlineStr"/>
+      <c r="V125" s="4" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -11620,11 +11926,16 @@
       </c>
       <c r="S126" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T126" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T126" s="2" t="inlineStr"/>
-      <c r="U126" s="4" t="inlineStr"/>
+      <c r="U126" s="2" t="inlineStr"/>
+      <c r="V126" s="4" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -11708,11 +12019,16 @@
       </c>
       <c r="S127" s="2" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="T127" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T127" s="2" t="inlineStr"/>
-      <c r="U127" s="4" t="inlineStr"/>
+      <c r="U127" s="2" t="inlineStr"/>
+      <c r="V127" s="4" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -11802,11 +12118,16 @@
       </c>
       <c r="S128" s="2" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="T128" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T128" s="2" t="inlineStr"/>
-      <c r="U128" s="4" t="inlineStr"/>
+      <c r="U128" s="2" t="inlineStr"/>
+      <c r="V128" s="4" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -11894,11 +12215,16 @@
       </c>
       <c r="S129" s="2" t="inlineStr">
         <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="T129" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T129" s="2" t="inlineStr"/>
-      <c r="U129" s="4" t="inlineStr"/>
+      <c r="U129" s="2" t="inlineStr"/>
+      <c r="V129" s="4" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -11981,13 +12307,14 @@
           <t>proyecto+licencia+DF+CFO a precio conjunto de 3.500; las fracciones de pago se perdieron en el texto (probablemente 1/3 cada una); en la casilla CIF pone la razón social</t>
         </is>
       </c>
-      <c r="S130" s="2" t="inlineStr">
+      <c r="S130" s="2" t="n"/>
+      <c r="T130" s="2" t="inlineStr">
         <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T130" s="2" t="inlineStr"/>
-      <c r="U130" s="4" t="inlineStr"/>
+      <c r="U130" s="2" t="inlineStr"/>
+      <c r="V130" s="4" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -12071,11 +12398,16 @@
       </c>
       <c r="S131" s="2" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="T131" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T131" s="2" t="inlineStr"/>
-      <c r="U131" s="4" t="inlineStr"/>
+      <c r="U131" s="2" t="inlineStr"/>
+      <c r="V131" s="4" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -12160,11 +12492,16 @@
       </c>
       <c r="S132" s="2" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="T132" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T132" s="2" t="inlineStr"/>
-      <c r="U132" s="4" t="inlineStr"/>
+      <c r="U132" s="2" t="inlineStr"/>
+      <c r="V132" s="4" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -12246,11 +12583,16 @@
       </c>
       <c r="S133" s="2" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="T133" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T133" s="2" t="inlineStr"/>
-      <c r="U133" s="4" t="inlineStr"/>
+      <c r="U133" s="2" t="inlineStr"/>
+      <c r="V133" s="4" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -12335,11 +12677,16 @@
       </c>
       <c r="S134" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T134" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T134" s="2" t="inlineStr"/>
-      <c r="U134" s="4" t="inlineStr"/>
+      <c r="U134" s="2" t="inlineStr"/>
+      <c r="V134" s="4" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -12429,11 +12776,16 @@
       </c>
       <c r="S135" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T135" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T135" s="2" t="inlineStr"/>
-      <c r="U135" s="4" t="inlineStr"/>
+      <c r="U135" s="2" t="inlineStr"/>
+      <c r="V135" s="4" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -12514,11 +12866,16 @@
       </c>
       <c r="S136" s="2" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="T136" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T136" s="2" t="inlineStr"/>
-      <c r="U136" s="4" t="inlineStr"/>
+      <c r="U136" s="2" t="inlineStr"/>
+      <c r="V136" s="4" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -12601,14 +12958,19 @@
       </c>
       <c r="S137" s="2" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="T137" s="2" t="inlineStr">
+        <is>
           <t>se asigna al final, con todas</t>
         </is>
       </c>
-      <c r="T137" s="2" t="inlineStr"/>
-      <c r="U137" s="4" t="inlineStr"/>
+      <c r="U137" s="2" t="inlineStr"/>
+      <c r="V137" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U137"/>
+  <autoFilter ref="A1:V137"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>